<commit_message>
Update issue where some nests were management status = N and management level = 1 or 2 Reran all nest survival analysis
</commit_message>
<xml_diff>
--- a/data/nest_issues_commented/MP_nest_data_issues_011025.xlsx
+++ b/data/nest_issues_commented/MP_nest_data_issues_011025.xlsx
@@ -132,45 +132,48 @@
     <t xml:space="preserve">dune</t>
   </si>
   <si>
+    <t xml:space="preserve">N</t>
+  </si>
+  <si>
+    <t xml:space="preserve">nodogssign</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-38.451469899999999</t>
+  </si>
+  <si>
+    <t xml:space="preserve">144.86279049999999</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Management type is not sufficient for making levels; </t>
+  </si>
+  <si>
+    <t xml:space="preserve">201314</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Koonya East</t>
+  </si>
+  <si>
+    <t xml:space="preserve">201314_Koonya East_2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">11112013</t>
+  </si>
+  <si>
+    <t xml:space="preserve">18112013</t>
+  </si>
+  <si>
+    <t xml:space="preserve">not specified</t>
+  </si>
+  <si>
     <t xml:space="preserve">Y</t>
   </si>
   <si>
-    <t xml:space="preserve">nodogssign</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-38.451469899999999</t>
-  </si>
-  <si>
-    <t xml:space="preserve">144.86279049999999</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MP</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Management type is not sufficient for making levels; </t>
-  </si>
-  <si>
-    <t xml:space="preserve">201314</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Koonya East</t>
-  </si>
-  <si>
-    <t xml:space="preserve">201314_Koonya East_2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">11112013</t>
-  </si>
-  <si>
-    <t xml:space="preserve">18112013</t>
-  </si>
-  <si>
-    <t xml:space="preserve">not specified</t>
-  </si>
-  <si>
     <t xml:space="preserve">signaccess,ropefence</t>
   </si>
   <si>
@@ -190,9 +193,6 @@
   </si>
   <si>
     <t xml:space="preserve">13022013</t>
-  </si>
-  <si>
-    <t xml:space="preserve">N</t>
   </si>
   <si>
     <t xml:space="preserve">permanentfence</t>
@@ -1065,10 +1065,10 @@
         <v>51</v>
       </c>
       <c r="I3" t="s">
-        <v>39</v>
+        <v>52</v>
       </c>
       <c r="J3" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="K3"/>
       <c r="L3"/>
@@ -1126,27 +1126,27 @@
         <v>44</v>
       </c>
       <c r="AF3" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B4" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C4" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D4" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E4" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="F4" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="G4" t="s">
         <v>37</v>
@@ -1155,7 +1155,7 @@
         <v>51</v>
       </c>
       <c r="I4" t="s">
-        <v>59</v>
+        <v>52</v>
       </c>
       <c r="J4" t="s">
         <v>60</v>
@@ -1214,7 +1214,7 @@
         <v>44</v>
       </c>
       <c r="AF4" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="5">
@@ -1243,7 +1243,7 @@
         <v>51</v>
       </c>
       <c r="I5" t="s">
-        <v>39</v>
+        <v>52</v>
       </c>
       <c r="J5" t="s">
         <v>65</v>
@@ -1306,7 +1306,7 @@
         <v>44</v>
       </c>
       <c r="AF5" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="6">
@@ -1335,7 +1335,7 @@
         <v>51</v>
       </c>
       <c r="I6" t="s">
-        <v>39</v>
+        <v>52</v>
       </c>
       <c r="J6" t="s">
         <v>65</v>
@@ -1394,7 +1394,7 @@
         <v>44</v>
       </c>
       <c r="AF6" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="7">
@@ -1423,7 +1423,7 @@
         <v>75</v>
       </c>
       <c r="I7" t="s">
-        <v>59</v>
+        <v>39</v>
       </c>
       <c r="J7" t="s">
         <v>26</v>
@@ -1488,7 +1488,7 @@
         <v>77</v>
       </c>
       <c r="AF7" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="8">
@@ -1517,7 +1517,7 @@
         <v>51</v>
       </c>
       <c r="I8" t="s">
-        <v>59</v>
+        <v>39</v>
       </c>
       <c r="J8" t="s">
         <v>26</v>
@@ -1576,7 +1576,7 @@
         <v>44</v>
       </c>
       <c r="AF8" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="9">
@@ -1605,10 +1605,10 @@
         <v>51</v>
       </c>
       <c r="I9" t="s">
-        <v>39</v>
+        <v>52</v>
       </c>
       <c r="J9" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="K9"/>
       <c r="L9"/>
@@ -1664,7 +1664,7 @@
         <v>44</v>
       </c>
       <c r="AF9" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="10">
@@ -1672,7 +1672,7 @@
         <v>68</v>
       </c>
       <c r="B10" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C10" t="s">
         <v>85</v>
@@ -1693,7 +1693,7 @@
         <v>51</v>
       </c>
       <c r="I10" t="s">
-        <v>59</v>
+        <v>39</v>
       </c>
       <c r="J10" t="s">
         <v>26</v>
@@ -1752,7 +1752,7 @@
         <v>44</v>
       </c>
       <c r="AF10" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="11">
@@ -1781,7 +1781,7 @@
         <v>51</v>
       </c>
       <c r="I11" t="s">
-        <v>59</v>
+        <v>39</v>
       </c>
       <c r="J11" t="s">
         <v>26</v>
@@ -1840,7 +1840,7 @@
         <v>44</v>
       </c>
       <c r="AF11" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="12">
@@ -1869,7 +1869,7 @@
         <v>51</v>
       </c>
       <c r="I12" t="s">
-        <v>59</v>
+        <v>39</v>
       </c>
       <c r="J12" t="s">
         <v>26</v>
@@ -1934,7 +1934,7 @@
         <v>92</v>
       </c>
       <c r="AF12" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="13">
@@ -1963,7 +1963,7 @@
         <v>51</v>
       </c>
       <c r="I13" t="s">
-        <v>39</v>
+        <v>52</v>
       </c>
       <c r="J13" t="s">
         <v>98</v>
@@ -2028,7 +2028,7 @@
         <v>92</v>
       </c>
       <c r="AF13" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="14">
@@ -2057,7 +2057,7 @@
         <v>51</v>
       </c>
       <c r="I14" t="s">
-        <v>59</v>
+        <v>39</v>
       </c>
       <c r="J14" t="s">
         <v>26</v>
@@ -2122,7 +2122,7 @@
         <v>103</v>
       </c>
       <c r="AF14" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="15">
@@ -2151,7 +2151,7 @@
         <v>51</v>
       </c>
       <c r="I15" t="s">
-        <v>59</v>
+        <v>39</v>
       </c>
       <c r="J15" t="s">
         <v>26</v>
@@ -2216,7 +2216,7 @@
         <v>107</v>
       </c>
       <c r="AF15" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="16">
@@ -2245,7 +2245,7 @@
         <v>51</v>
       </c>
       <c r="I16" t="s">
-        <v>59</v>
+        <v>39</v>
       </c>
       <c r="J16" t="s">
         <v>26</v>
@@ -2310,7 +2310,7 @@
         <v>111</v>
       </c>
       <c r="AF16" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="17">
@@ -2339,7 +2339,7 @@
         <v>51</v>
       </c>
       <c r="I17" t="s">
-        <v>39</v>
+        <v>52</v>
       </c>
       <c r="J17" t="s">
         <v>116</v>
@@ -2404,7 +2404,7 @@
         <v>117</v>
       </c>
       <c r="AF17" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="18">
@@ -2433,7 +2433,7 @@
         <v>51</v>
       </c>
       <c r="I18" t="s">
-        <v>39</v>
+        <v>52</v>
       </c>
       <c r="J18" t="s">
         <v>116</v>
@@ -2492,7 +2492,7 @@
         <v>44</v>
       </c>
       <c r="AF18" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="19">
@@ -2521,7 +2521,7 @@
         <v>51</v>
       </c>
       <c r="I19" t="s">
-        <v>59</v>
+        <v>39</v>
       </c>
       <c r="J19" t="s">
         <v>26</v>
@@ -2582,7 +2582,7 @@
         <v>44</v>
       </c>
       <c r="AF19" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="20">
@@ -2611,7 +2611,7 @@
         <v>51</v>
       </c>
       <c r="I20" t="s">
-        <v>59</v>
+        <v>39</v>
       </c>
       <c r="J20" t="s">
         <v>26</v>
@@ -2670,7 +2670,7 @@
         <v>44</v>
       </c>
       <c r="AF20" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="21">
@@ -2699,7 +2699,7 @@
         <v>51</v>
       </c>
       <c r="I21" t="s">
-        <v>59</v>
+        <v>39</v>
       </c>
       <c r="J21" t="s">
         <v>26</v>
@@ -2760,7 +2760,7 @@
         <v>44</v>
       </c>
       <c r="AF21" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="22">
@@ -2789,7 +2789,7 @@
         <v>51</v>
       </c>
       <c r="I22" t="s">
-        <v>59</v>
+        <v>39</v>
       </c>
       <c r="J22" t="s">
         <v>26</v>
@@ -2850,7 +2850,7 @@
         <v>44</v>
       </c>
       <c r="AF22" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="23">
@@ -2879,7 +2879,7 @@
         <v>51</v>
       </c>
       <c r="I23" t="s">
-        <v>39</v>
+        <v>52</v>
       </c>
       <c r="J23" t="s">
         <v>116</v>
@@ -2944,7 +2944,7 @@
         <v>77</v>
       </c>
       <c r="AF23" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="24">
@@ -2973,7 +2973,7 @@
         <v>51</v>
       </c>
       <c r="I24" t="s">
-        <v>59</v>
+        <v>39</v>
       </c>
       <c r="J24" t="s">
         <v>26</v>
@@ -3032,7 +3032,7 @@
         <v>44</v>
       </c>
       <c r="AF24" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="25">
@@ -3061,7 +3061,7 @@
         <v>51</v>
       </c>
       <c r="I25" t="s">
-        <v>39</v>
+        <v>52</v>
       </c>
       <c r="J25" t="s">
         <v>116</v>
@@ -3122,7 +3122,7 @@
         <v>44</v>
       </c>
       <c r="AF25" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="26">
@@ -3151,7 +3151,7 @@
         <v>51</v>
       </c>
       <c r="I26" t="s">
-        <v>59</v>
+        <v>39</v>
       </c>
       <c r="J26" t="s">
         <v>26</v>
@@ -3210,7 +3210,7 @@
         <v>44</v>
       </c>
       <c r="AF26" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="27">
@@ -3239,7 +3239,7 @@
         <v>51</v>
       </c>
       <c r="I27" t="s">
-        <v>59</v>
+        <v>39</v>
       </c>
       <c r="J27" t="s">
         <v>26</v>
@@ -3304,7 +3304,7 @@
         <v>156</v>
       </c>
       <c r="AF27" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="28">
@@ -3333,7 +3333,7 @@
         <v>51</v>
       </c>
       <c r="I28" t="s">
-        <v>59</v>
+        <v>39</v>
       </c>
       <c r="J28" t="s">
         <v>26</v>
@@ -3402,7 +3402,7 @@
         <v>164</v>
       </c>
       <c r="AF28" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="29">
@@ -3431,7 +3431,7 @@
         <v>51</v>
       </c>
       <c r="I29" t="s">
-        <v>59</v>
+        <v>39</v>
       </c>
       <c r="J29" t="s">
         <v>26</v>
@@ -3490,7 +3490,7 @@
         <v>44</v>
       </c>
       <c r="AF29" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
   </sheetData>

</xml_diff>